<commit_message>
Add Skalbmierz to 2026 season standings
</commit_message>
<xml_diff>
--- a/data/Klasyfikacja_generalna_Tyberian_Team_2026.xlsx
+++ b/data/Klasyfikacja_generalna_Tyberian_Team_2026.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klasyfikacja" sheetId="1" r:id="Rc01a7969faa94e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Obliczenia" sheetId="2" r:id="Rc5b1bc21f7f547da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wyniki zawodów" sheetId="3" r:id="R386bf36608744df8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawody" sheetId="4" r:id="R5b0312df97944fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawodnicy" sheetId="5" r:id="Re024210feb5e42e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrukcja" sheetId="6" r:id="R54b6b7350c9a4cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klasyfikacja" sheetId="1" r:id="Rbeb5276e34194628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Obliczenia" sheetId="2" r:id="Rea323cc69d5b4d88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wyniki zawodów" sheetId="3" r:id="R0a328613dc2d43d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawody" sheetId="4" r:id="Reffe2169ae324a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawodnicy" sheetId="5" r:id="Rabaf61ef93b049e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrukcja" sheetId="6" r:id="R4352c38930be4cbd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -819,8 +819,8 @@
       </x:c>
       <x:c r="N5" s="14" t="str">
         <x:v>11
-Slot 11
-</x:v>
+Skalbmierz
+09.08.2026</x:v>
       </x:c>
       <x:c r="O5" s="14" t="str">
         <x:v>12
@@ -1206,7 +1206,7 @@
       </x:c>
       <x:c r="C9" s="17" t="n">
         <x:f>IF(B9="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B9,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D9" s="28" t="n">
         <x:f>IF(B9="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B9,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1250,7 +1250,7 @@
       </x:c>
       <x:c r="N9" s="28" t="n">
         <x:f>IF(B9="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B9,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O9" s="28" t="n">
         <x:f>IF(B9="","",INDEX(Obliczenia!$O$6:$O$55,MATCH(B9,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1290,15 +1290,15 @@
       </x:c>
       <x:c r="X9" s="17" t="n">
         <x:f>IF(B9="","",INDEX(Obliczenia!$X$6:$X$55,MATCH(B9,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="Y9" s="29" t="n">
         <x:f>IF(B9="","",INDEX(Obliczenia!$Y$6:$Y$55,MATCH(B9,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="Z9" s="30" t="n">
         <x:f>IF(B9="","",INDEX(Obliczenia!$Z$6:$Z$55,MATCH(B9,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1630,7 +1630,7 @@
       </x:c>
       <x:c r="C13" s="17" t="n">
         <x:f>IF(B13="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B13,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D13" s="28" t="n">
         <x:f>IF(B13="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B13,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1674,7 +1674,7 @@
       </x:c>
       <x:c r="N13" s="28" t="n">
         <x:f>IF(B13="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B13,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O13" s="28" t="n">
         <x:f>IF(B13="","",INDEX(Obliczenia!$O$6:$O$55,MATCH(B13,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1714,15 +1714,15 @@
       </x:c>
       <x:c r="X13" s="17" t="n">
         <x:f>IF(B13="","",INDEX(Obliczenia!$X$6:$X$55,MATCH(B13,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>12</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="Y13" s="29" t="n">
         <x:f>IF(B13="","",INDEX(Obliczenia!$Y$6:$Y$55,MATCH(B13,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="Z13" s="30" t="n">
         <x:f>IF(B13="","",INDEX(Obliczenia!$Z$6:$Z$55,MATCH(B13,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1732,19 +1732,19 @@
       </x:c>
       <x:c r="B14" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,9),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-        <x:v>Krzysztof Kacnerski</x:v>
+        <x:v>Tomasz Lademann</x:v>
       </x:c>
       <x:c r="C14" s="17" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$E$6:$E$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$F$6:$F$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1756,7 +1756,7 @@
       </x:c>
       <x:c r="H14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$H$6:$H$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$I$6:$I$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1768,7 +1768,7 @@
       </x:c>
       <x:c r="K14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$K$6:$K$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$L$6:$L$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1776,11 +1776,11 @@
       </x:c>
       <x:c r="M14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$M$6:$M$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O14" s="28" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$O$6:$O$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1820,11 +1820,11 @@
       </x:c>
       <x:c r="X14" s="17" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$X$6:$X$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="Y14" s="29" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$Y$6:$Y$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="Z14" s="30" t="n">
         <x:f>IF(B14="","",INDEX(Obliczenia!$Z$6:$Z$55,MATCH(B14,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1838,19 +1838,19 @@
       </x:c>
       <x:c r="B15" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,10),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-        <x:v>Marcin Schabowski</x:v>
+        <x:v>Krzysztof Kacnerski</x:v>
       </x:c>
       <x:c r="C15" s="17" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$E$6:$E$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$F$6:$F$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1862,7 +1862,7 @@
       </x:c>
       <x:c r="H15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$H$6:$H$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$I$6:$I$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1874,7 +1874,7 @@
       </x:c>
       <x:c r="K15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$K$6:$K$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$L$6:$L$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1882,7 +1882,7 @@
       </x:c>
       <x:c r="M15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$M$6:$M$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N15" s="28" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1926,11 +1926,11 @@
       </x:c>
       <x:c r="X15" s="17" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$X$6:$X$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Y15" s="29" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$Y$6:$Y$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="Z15" s="30" t="n">
         <x:f>IF(B15="","",INDEX(Obliczenia!$Z$6:$Z$55,MATCH(B15,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1940,15 +1940,15 @@
     <x:row r="16">
       <x:c r="A16" s="33" t="n">
         <x:f>IF(B16="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y16))</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B16" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,11),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-        <x:v>Mariusz Pachut</x:v>
+        <x:v>Marcin Schabowski</x:v>
       </x:c>
       <x:c r="C16" s="17" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1956,7 +1956,7 @@
       </x:c>
       <x:c r="E16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$E$6:$E$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$F$6:$F$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1964,7 +1964,7 @@
       </x:c>
       <x:c r="G16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$G$6:$G$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$H$6:$H$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -1984,11 +1984,11 @@
       </x:c>
       <x:c r="L16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$L$6:$L$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$M$6:$M$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N16" s="28" t="n">
         <x:f>IF(B16="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B16,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2046,15 +2046,15 @@
     <x:row r="17">
       <x:c r="A17" s="33" t="n">
         <x:f>IF(B17="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y17))</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,12),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-        <x:v>Adam Wądołowski</x:v>
+        <x:v>Mariusz Pachut</x:v>
       </x:c>
       <x:c r="C17" s="17" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2062,7 +2062,7 @@
       </x:c>
       <x:c r="E17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$E$6:$E$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$F$6:$F$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2070,7 +2070,7 @@
       </x:c>
       <x:c r="G17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$G$6:$G$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$H$6:$H$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2078,7 +2078,7 @@
       </x:c>
       <x:c r="I17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$I$6:$I$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$J$6:$J$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2086,15 +2086,15 @@
       </x:c>
       <x:c r="K17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$K$6:$K$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$L$6:$L$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$M$6:$M$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N17" s="28" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2138,11 +2138,11 @@
       </x:c>
       <x:c r="X17" s="17" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$X$6:$X$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Y17" s="29" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$Y$6:$Y$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="Z17" s="30" t="n">
         <x:f>IF(B17="","",INDEX(Obliczenia!$Z$6:$Z$55,MATCH(B17,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2152,15 +2152,15 @@
     <x:row r="18">
       <x:c r="A18" s="33" t="n">
         <x:f>IF(B18="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y18))</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B18" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,13),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-        <x:v>Tomasz Lademann</x:v>
+        <x:v>Adam Wądołowski</x:v>
       </x:c>
       <x:c r="C18" s="17" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D18" s="28" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2168,7 +2168,7 @@
       </x:c>
       <x:c r="E18" s="28" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$E$6:$E$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="28" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$F$6:$F$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2184,7 +2184,7 @@
       </x:c>
       <x:c r="I18" s="28" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$I$6:$I$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J18" s="28" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$J$6:$J$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2192,7 +2192,7 @@
       </x:c>
       <x:c r="K18" s="28" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$K$6:$K$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L18" s="28" t="n">
         <x:f>IF(B18="","",INDEX(Obliczenia!$L$6:$L$55,MATCH(B18,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2262,11 +2262,11 @@
       </x:c>
       <x:c r="B19" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,14),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-        <x:v>Przemysław Marczewski</x:v>
+        <x:v>Michał Maruszewski</x:v>
       </x:c>
       <x:c r="C19" s="17" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D19" s="28" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2282,7 +2282,7 @@
       </x:c>
       <x:c r="G19" s="28" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$G$6:$G$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H19" s="28" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$H$6:$H$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2294,7 +2294,7 @@
       </x:c>
       <x:c r="J19" s="28" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$J$6:$J$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K19" s="28" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$K$6:$K$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2310,7 +2310,7 @@
       </x:c>
       <x:c r="N19" s="28" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O19" s="28" t="n">
         <x:f>IF(B19="","",INDEX(Obliczenia!$O$6:$O$55,MATCH(B19,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2364,11 +2364,11 @@
     <x:row r="20">
       <x:c r="A20" s="33" t="n">
         <x:f>IF(B20="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y20))</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B20" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,15),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-        <x:v>Michał Maruszewski</x:v>
+        <x:v>Przemysław Marczewski</x:v>
       </x:c>
       <x:c r="C20" s="17" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2388,7 +2388,7 @@
       </x:c>
       <x:c r="G20" s="28" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$G$6:$G$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H20" s="28" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$H$6:$H$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2400,7 +2400,7 @@
       </x:c>
       <x:c r="J20" s="28" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$J$6:$J$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K20" s="28" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$K$6:$K$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2456,11 +2456,11 @@
       </x:c>
       <x:c r="X20" s="17" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$X$6:$X$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Y20" s="29" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$Y$6:$Y$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Z20" s="30" t="n">
         <x:f>IF(B20="","",INDEX(Obliczenia!$Z$6:$Z$55,MATCH(B20,Obliczenia!$B$6:$B$55,0)))</x:f>
@@ -2468,83 +2468,109 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="33" t="str">
+      <x:c r="A21" s="33" t="n">
         <x:f>IF(B21="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y21))</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
         <x:f>IFERROR(INDEX(Obliczenia!$B$6:$B$55,MATCH(LARGE(Obliczenia!$AA$6:$AA$55,16),Obliczenia!$AA$6:$AA$55,0)),"")</x:f>
-      </x:c>
-      <x:c r="C21" s="17" t="str">
+        <x:v>Michał Sajdak</x:v>
+      </x:c>
+      <x:c r="C21" s="17" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$C$6:$C$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="D21" s="28" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$D$6:$D$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="E21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$E$6:$E$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="F21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$F$6:$F$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="G21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$G$6:$G$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="H21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$H$6:$H$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="I21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$I$6:$I$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="J21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$J$6:$J$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="K21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$K$6:$K$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="L21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$L$6:$L$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="M21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$M$6:$M$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="N21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$N$6:$N$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="O21" s="28" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$O$6:$O$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="P21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$P$6:$P$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="Q21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$Q$6:$Q$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="R21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$R$6:$R$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="S21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$S$6:$S$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="T21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$T$6:$T$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="U21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$U$6:$U$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="V21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$V$6:$V$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="W21" s="28" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W21" s="28" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$W$6:$W$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="X21" s="17" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X21" s="17" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$X$6:$X$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="Y21" s="29" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y21" s="29" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$Y$6:$Y$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
-      </x:c>
-      <x:c r="Z21" s="30" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Z21" s="30" t="n">
         <x:f>IF(B21="","",INDEX(Obliczenia!$Z$6:$Z$55,MATCH(B21,Obliczenia!$B$6:$B$55,0)))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5689,8 +5715,8 @@
       </x:c>
       <x:c r="N5" s="14" t="str">
         <x:v>11
-Slot 11
-</x:v>
+Skalbmierz
+09.08.2026</x:v>
       </x:c>
       <x:c r="O5" s="14" t="str">
         <x:v>12
@@ -5753,7 +5779,7 @@
     <x:row r="6">
       <x:c r="A6" s="17" t="n">
         <x:f>IF(B6="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y6))</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
         <x:f>IF(COUNTIF('Wyniki zawodów'!$F$6:$F$205,Zawodnicy!A6)=0,"",Zawodnicy!A6)</x:f>
@@ -5981,7 +6007,7 @@
       </x:c>
       <x:c r="C8" s="17" t="n">
         <x:f>IF(B8="","",COUNTIF('Wyniki zawodów'!$F$6:$F$205,B8))</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="28" t="n">
         <x:f>IF($B8="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B8,'Wyniki zawodów'!$A$6:$A$205,D$4))</x:f>
@@ -6025,7 +6051,7 @@
       </x:c>
       <x:c r="N8" s="28" t="n">
         <x:f>IF($B8="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B8,'Wyniki zawodów'!$A$6:$A$205,N$4))</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O8" s="28" t="n">
         <x:f>IF($B8="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B8,'Wyniki zawodów'!$A$6:$A$205,O$4))</x:f>
@@ -6065,19 +6091,19 @@
       </x:c>
       <x:c r="X8" s="17" t="n">
         <x:f>IF(B8="","",SUM(D8:W8))</x:f>
-        <x:v>12</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="Y8" s="29" t="n">
         <x:f>IF(B8="","",LARGE(D8:W8,1)+LARGE(D8:W8,2)+LARGE(D8:W8,3)+LARGE(D8:W8,4))</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="Z8" s="17" t="n">
         <x:f>IF(B8="","",X8-Y8)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AA8" s="17" t="n">
         <x:f>IF(B8="",0,Y8*1000+(100-ROW()))</x:f>
-        <x:v>10092</x:v>
+        <x:v>11092</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6609,7 +6635,7 @@
     <x:row r="14">
       <x:c r="A14" s="17" t="n">
         <x:f>IF(B14="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y14))</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B14" s="17" t="str">
         <x:f>IF(COUNTIF('Wyniki zawodów'!$F$6:$F$205,Zawodnicy!A14)=0,"",Zawodnicy!A14)</x:f>
@@ -6829,7 +6855,7 @@
     <x:row r="16">
       <x:c r="A16" s="17" t="n">
         <x:f>IF(B16="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y16))</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B16" s="17" t="str">
         <x:f>IF(COUNTIF('Wyniki zawodów'!$F$6:$F$205,Zawodnicy!A16)=0,"",Zawodnicy!A16)</x:f>
@@ -6947,7 +6973,7 @@
       </x:c>
       <x:c r="C17" s="17" t="n">
         <x:f>IF(B17="","",COUNTIF('Wyniki zawodów'!$F$6:$F$205,B17))</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D17" s="28" t="n">
         <x:f>IF($B17="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B17,'Wyniki zawodów'!$A$6:$A$205,D$4))</x:f>
@@ -6991,7 +7017,7 @@
       </x:c>
       <x:c r="N17" s="28" t="n">
         <x:f>IF($B17="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B17,'Wyniki zawodów'!$A$6:$A$205,N$4))</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O17" s="28" t="n">
         <x:f>IF($B17="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B17,'Wyniki zawodów'!$A$6:$A$205,O$4))</x:f>
@@ -7031,25 +7057,25 @@
       </x:c>
       <x:c r="X17" s="17" t="n">
         <x:f>IF(B17="","",SUM(D17:W17))</x:f>
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="Y17" s="29" t="n">
         <x:f>IF(B17="","",LARGE(D17:W17,1)+LARGE(D17:W17,2)+LARGE(D17:W17,3)+LARGE(D17:W17,4))</x:f>
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="Z17" s="17" t="n">
         <x:f>IF(B17="","",X17-Y17)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AA17" s="17" t="n">
         <x:f>IF(B17="",0,Y17*1000+(100-ROW()))</x:f>
-        <x:v>15083</x:v>
+        <x:v>17083</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="17" t="n">
         <x:f>IF(B18="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y18))</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B18" s="17" t="str">
         <x:f>IF(COUNTIF('Wyniki zawodów'!$F$6:$F$205,Zawodnicy!A18)=0,"",Zawodnicy!A18)</x:f>
@@ -7159,7 +7185,7 @@
     <x:row r="19">
       <x:c r="A19" s="17" t="n">
         <x:f>IF(B19="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y19))</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
         <x:f>IF(COUNTIF('Wyniki zawodów'!$F$6:$F$205,Zawodnicy!A19)=0,"",Zawodnicy!A19)</x:f>
@@ -7167,7 +7193,7 @@
       </x:c>
       <x:c r="C19" s="17" t="n">
         <x:f>IF(B19="","",COUNTIF('Wyniki zawodów'!$F$6:$F$205,B19))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D19" s="28" t="n">
         <x:f>IF($B19="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B19,'Wyniki zawodów'!$A$6:$A$205,D$4))</x:f>
@@ -7211,7 +7237,7 @@
       </x:c>
       <x:c r="N19" s="28" t="n">
         <x:f>IF($B19="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B19,'Wyniki zawodów'!$A$6:$A$205,N$4))</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O19" s="28" t="n">
         <x:f>IF($B19="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B19,'Wyniki zawodów'!$A$6:$A$205,O$4))</x:f>
@@ -7251,11 +7277,11 @@
       </x:c>
       <x:c r="X19" s="17" t="n">
         <x:f>IF(B19="","",SUM(D19:W19))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Y19" s="29" t="n">
         <x:f>IF(B19="","",LARGE(D19:W19,1)+LARGE(D19:W19,2)+LARGE(D19:W19,3)+LARGE(D19:W19,4))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="Z19" s="17" t="n">
         <x:f>IF(B19="","",X19-Y19)</x:f>
@@ -7263,7 +7289,7 @@
       </x:c>
       <x:c r="AA19" s="17" t="n">
         <x:f>IF(B19="",0,Y19*1000+(100-ROW()))</x:f>
-        <x:v>1081</x:v>
+        <x:v>2081</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -7813,7 +7839,7 @@
     <x:row r="25">
       <x:c r="A25" s="17" t="n">
         <x:f>IF(B25="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y25))</x:f>
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B25" s="17" t="str">
         <x:f>IF(COUNTIF('Wyniki zawodów'!$F$6:$F$205,Zawodnicy!A25)=0,"",Zawodnicy!A25)</x:f>
@@ -7821,7 +7847,7 @@
       </x:c>
       <x:c r="C25" s="17" t="n">
         <x:f>IF(B25="","",COUNTIF('Wyniki zawodów'!$F$6:$F$205,B25))</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D25" s="28" t="n">
         <x:f>IF($B25="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B25,'Wyniki zawodów'!$A$6:$A$205,D$4))</x:f>
@@ -7865,7 +7891,7 @@
       </x:c>
       <x:c r="N25" s="28" t="n">
         <x:f>IF($B25="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B25,'Wyniki zawodów'!$A$6:$A$205,N$4))</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O25" s="28" t="n">
         <x:f>IF($B25="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B25,'Wyniki zawodów'!$A$6:$A$205,O$4))</x:f>
@@ -7905,11 +7931,11 @@
       </x:c>
       <x:c r="X25" s="17" t="n">
         <x:f>IF(B25="","",SUM(D25:W25))</x:f>
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="Y25" s="29" t="n">
         <x:f>IF(B25="","",LARGE(D25:W25,1)+LARGE(D25:W25,2)+LARGE(D25:W25,3)+LARGE(D25:W25,4))</x:f>
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="Z25" s="17" t="n">
         <x:f>IF(B25="","",X25-Y25)</x:f>
@@ -7917,18 +7943,21 @@
       </x:c>
       <x:c r="AA25" s="17" t="n">
         <x:f>IF(B25="",0,Y25*1000+(100-ROW()))</x:f>
-        <x:v>3075</x:v>
+        <x:v>7075</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="17" t="str">
+      <x:c r="A26" s="17" t="n">
         <x:f>IF(B26="","",1+COUNTIF($Y$6:$Y$55,"&gt;"&amp;Y26))</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B26" s="17" t="str">
         <x:f>IF(COUNTIF('Wyniki zawodów'!$F$6:$F$205,Zawodnicy!A26)=0,"",Zawodnicy!A26)</x:f>
-      </x:c>
-      <x:c r="C26" s="17" t="str">
+        <x:v>Michał Sajdak</x:v>
+      </x:c>
+      <x:c r="C26" s="17" t="n">
         <x:f>IF(B26="","",COUNTIF('Wyniki zawodów'!$F$6:$F$205,B26))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D26" s="28" t="n">
         <x:f>IF($B26="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B26,'Wyniki zawodów'!$A$6:$A$205,D$4))</x:f>
@@ -7972,7 +8001,7 @@
       </x:c>
       <x:c r="N26" s="28" t="n">
         <x:f>IF($B26="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B26,'Wyniki zawodów'!$A$6:$A$205,N$4))</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O26" s="28" t="n">
         <x:f>IF($B26="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B26,'Wyniki zawodów'!$A$6:$A$205,O$4))</x:f>
@@ -8010,18 +8039,21 @@
         <x:f>IF($B26="",0,SUMIFS('Wyniki zawodów'!$G$6:$G$205,'Wyniki zawodów'!$F$6:$F$205,$B26,'Wyniki zawodów'!$A$6:$A$205,W$4))</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="X26" s="17" t="str">
+      <x:c r="X26" s="17" t="n">
         <x:f>IF(B26="","",SUM(D26:W26))</x:f>
-      </x:c>
-      <x:c r="Y26" s="29" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Y26" s="29" t="n">
         <x:f>IF(B26="","",LARGE(D26:W26,1)+LARGE(D26:W26,2)+LARGE(D26:W26,3)+LARGE(D26:W26,4))</x:f>
-      </x:c>
-      <x:c r="Z26" s="17" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Z26" s="17" t="n">
         <x:f>IF(B26="","",X26-Y26)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AA26" s="17" t="n">
         <x:f>IF(B26="",0,Y26*1000+(100-ROW()))</x:f>
-        <x:v>0</x:v>
+        <x:v>2074</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -12631,89 +12663,149 @@
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="18" t="str"/>
-      <x:c r="B56" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A56,Zawody!$A$6:$F$25,2,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="C56" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A56,Zawody!$A$6:$F$25,3,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="D56" s="18" t="str"/>
-      <x:c r="E56" s="17" t="str"/>
-      <x:c r="F56" s="17" t="str"/>
-      <x:c r="G56" s="25" t="str">
-        <x:f>IF(OR(A56="",D56=""),"",IF(AND(D56&gt;=1,D56&lt;=5),6-D56,0))</x:f>
-      </x:c>
-      <x:c r="H56" s="22" t="str"/>
-      <x:c r="I56" s="17" t="str"/>
+      <x:c r="A56" s="19" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B56" s="20" t="str">
+        <x:v>09.08.2026</x:v>
+      </x:c>
+      <x:c r="C56" s="20" t="str">
+        <x:v>Skalbmierz</x:v>
+      </x:c>
+      <x:c r="D56" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E56" s="26" t="str">
+        <x:v>MARCIN STANKIEWICZ</x:v>
+      </x:c>
+      <x:c r="F56" s="26" t="str">
+        <x:v>Marcin Stankiewicz</x:v>
+      </x:c>
+      <x:c r="G56" s="25" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H56" s="24" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="I56" s="20" t="str">
+        <x:v>Podsumowanie Skalbmierz 09.08.2026 (HTML)</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="18" t="str"/>
-      <x:c r="B57" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A57,Zawody!$A$6:$F$25,2,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="C57" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A57,Zawody!$A$6:$F$25,3,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="D57" s="18" t="str"/>
-      <x:c r="E57" s="17" t="str"/>
-      <x:c r="F57" s="17" t="str"/>
-      <x:c r="G57" s="25" t="str">
-        <x:f>IF(OR(A57="",D57=""),"",IF(AND(D57&gt;=1,D57&lt;=5),6-D57,0))</x:f>
-      </x:c>
-      <x:c r="H57" s="22" t="str"/>
-      <x:c r="I57" s="17" t="str"/>
+      <x:c r="A57" s="19" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B57" s="20" t="str">
+        <x:v>09.08.2026</x:v>
+      </x:c>
+      <x:c r="C57" s="20" t="str">
+        <x:v>Skalbmierz</x:v>
+      </x:c>
+      <x:c r="D57" s="19" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E57" s="26" t="str">
+        <x:v>TOMASZ LADEMANN</x:v>
+      </x:c>
+      <x:c r="F57" s="26" t="str">
+        <x:v>Tomasz Lademann</x:v>
+      </x:c>
+      <x:c r="G57" s="25" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H57" s="24" t="n">
+        <x:v>23.5</x:v>
+      </x:c>
+      <x:c r="I57" s="20" t="str">
+        <x:v>Podsumowanie Skalbmierz 09.08.2026 (HTML)</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="18" t="str"/>
-      <x:c r="B58" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A58,Zawody!$A$6:$F$25,2,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="C58" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A58,Zawody!$A$6:$F$25,3,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="D58" s="18" t="str"/>
-      <x:c r="E58" s="17" t="str"/>
-      <x:c r="F58" s="17" t="str"/>
-      <x:c r="G58" s="25" t="str">
-        <x:f>IF(OR(A58="",D58=""),"",IF(AND(D58&gt;=1,D58&lt;=5),6-D58,0))</x:f>
-      </x:c>
-      <x:c r="H58" s="22" t="str"/>
-      <x:c r="I58" s="17" t="str"/>
+      <x:c r="A58" s="19" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B58" s="20" t="str">
+        <x:v>09.08.2026</x:v>
+      </x:c>
+      <x:c r="C58" s="20" t="str">
+        <x:v>Skalbmierz</x:v>
+      </x:c>
+      <x:c r="D58" s="19" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E58" s="26" t="str">
+        <x:v>BARTOSZ POSTÓJ</x:v>
+      </x:c>
+      <x:c r="F58" s="26" t="str">
+        <x:v>Bartosz Postój</x:v>
+      </x:c>
+      <x:c r="G58" s="25" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H58" s="24" t="n">
+        <x:v>19.5</x:v>
+      </x:c>
+      <x:c r="I58" s="20" t="str">
+        <x:v>Podsumowanie Skalbmierz 09.08.2026 (HTML)</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="18" t="str"/>
-      <x:c r="B59" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A59,Zawody!$A$6:$F$25,2,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="C59" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A59,Zawody!$A$6:$F$25,3,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="D59" s="18" t="str"/>
-      <x:c r="E59" s="17" t="str"/>
-      <x:c r="F59" s="17" t="str"/>
-      <x:c r="G59" s="25" t="str">
-        <x:f>IF(OR(A59="",D59=""),"",IF(AND(D59&gt;=1,D59&lt;=5),6-D59,0))</x:f>
-      </x:c>
-      <x:c r="H59" s="22" t="str"/>
-      <x:c r="I59" s="17" t="str"/>
+      <x:c r="A59" s="19" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B59" s="20" t="str">
+        <x:v>09.08.2026</x:v>
+      </x:c>
+      <x:c r="C59" s="20" t="str">
+        <x:v>Skalbmierz</x:v>
+      </x:c>
+      <x:c r="D59" s="19" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E59" s="26" t="str">
+        <x:v>MICHAŁ SAJDAK</x:v>
+      </x:c>
+      <x:c r="F59" s="26" t="str">
+        <x:v>Michał Sajdak</x:v>
+      </x:c>
+      <x:c r="G59" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H59" s="24" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="I59" s="20" t="str">
+        <x:v>Podsumowanie Skalbmierz 09.08.2026 (HTML)</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="18" t="str"/>
-      <x:c r="B60" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A60,Zawody!$A$6:$F$25,2,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="C60" s="17" t="str">
-        <x:f>IFERROR(VLOOKUP(A60,Zawody!$A$6:$F$25,3,FALSE),"")</x:f>
-      </x:c>
-      <x:c r="D60" s="18" t="str"/>
-      <x:c r="E60" s="17" t="str"/>
-      <x:c r="F60" s="17" t="str"/>
-      <x:c r="G60" s="25" t="str">
-        <x:f>IF(OR(A60="",D60=""),"",IF(AND(D60&gt;=1,D60&lt;=5),6-D60,0))</x:f>
-      </x:c>
-      <x:c r="H60" s="22" t="str"/>
-      <x:c r="I60" s="17" t="str"/>
+      <x:c r="A60" s="19" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B60" s="20" t="str">
+        <x:v>09.08.2026</x:v>
+      </x:c>
+      <x:c r="C60" s="20" t="str">
+        <x:v>Skalbmierz</x:v>
+      </x:c>
+      <x:c r="D60" s="19" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E60" s="26" t="str">
+        <x:v>MICHAŁ MARUSZEWSKI</x:v>
+      </x:c>
+      <x:c r="F60" s="26" t="str">
+        <x:v>Michał Maruszewski</x:v>
+      </x:c>
+      <x:c r="G60" s="25" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H60" s="24" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I60" s="20" t="str">
+        <x:v>Podsumowanie Skalbmierz 09.08.2026 (HTML)</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="18" t="str"/>
@@ -15233,42 +15325,42 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="C2" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="D2" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="E2" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="F2" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="C3" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="E3" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
       <x:c r="F3" s="8" t="str">
-        <x:v>Dziesięć imprez jest już wpisanych chronologicznie. Wiersze 16-25 pozostają gotowe na kolejne zawody sezonu 2026.</x:v>
+        <x:v>Wpisano chronologicznie 11 imprez. Pozostałe wiersze są gotowe na kolejne zawody sezonu 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="44" customHeight="1">
@@ -15492,16 +15584,24 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="18" t="n">
+      <x:c r="A16" s="19" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B16" s="17"/>
-      <x:c r="C16" s="17" t="str"/>
-      <x:c r="D16" s="17" t="str"/>
-      <x:c r="E16" s="17" t="str">
-        <x:v>Planowane</x:v>
-      </x:c>
-      <x:c r="F16" s="17" t="str"/>
+      <x:c r="B16" s="20" t="str">
+        <x:v>09.08.2026</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="str">
+        <x:v>Skalbmierz</x:v>
+      </x:c>
+      <x:c r="D16" s="20" t="str">
+        <x:v>Skalbmierz · 09.08.2026</x:v>
+      </x:c>
+      <x:c r="E16" s="20" t="str">
+        <x:v>Rozegrane</x:v>
+      </x:c>
+      <x:c r="F16" s="20" t="str">
+        <x:v>Podsumowanie Skalbmierz 09.08.2026 (HTML)</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="18" t="n">
@@ -16107,12 +16207,18 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="17" t="str"/>
-      <x:c r="B26" s="17" t="str"/>
-      <x:c r="C26" s="17" t="str"/>
-      <x:c r="D26" s="17" t="str"/>
-      <x:c r="E26" s="17" t="str"/>
-      <x:c r="F26" s="17" t="str"/>
+      <x:c r="A26" s="20" t="str">
+        <x:v>Michał Sajdak</x:v>
+      </x:c>
+      <x:c r="B26" s="20" t="str">
+        <x:v>Tak</x:v>
+      </x:c>
+      <x:c r="C26" s="20" t="str"/>
+      <x:c r="D26" s="20" t="str"/>
+      <x:c r="E26" s="20" t="str"/>
+      <x:c r="F26" s="20" t="str">
+        <x:v>Dane profilu do uzupełnienia.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="17" t="str"/>

</xml_diff>